<commit_message>
Update ratings 2026-07-03 13:00
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -538,6 +538,33 @@
       </c>
       <c r="G2">
         <f>IF(D2&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C3" t="n">
+        <v>9747</v>
+      </c>
+      <c r="D3" t="n">
+        <v>40</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1">
+        <f>IFERROR(E3/D3,0)</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>IF(D3&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-07-04 13:00
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -565,6 +565,33 @@
       </c>
       <c r="G3">
         <f>IF(D3&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9777</v>
+      </c>
+      <c r="D4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
+        <f>IFERROR(E4/D4,0)</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>IF(D4&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-07-05 13:00
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -592,6 +592,33 @@
       </c>
       <c r="G4">
         <f>IF(D4&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C5" t="n">
+        <v>9793</v>
+      </c>
+      <c r="D5" t="n">
+        <v>16</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1">
+        <f>IFERROR(E5/D5,0)</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>IF(D5&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-07-06 13:00
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,6 +619,33 @@
       </c>
       <c r="G5">
         <f>IF(D5&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>9823</v>
+      </c>
+      <c r="D6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1">
+        <f>IFERROR(E6/D6,0)</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>IF(D6&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-07-07 13:00
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -646,6 +646,33 @@
       </c>
       <c r="G6">
         <f>IF(D6&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>9914</v>
+      </c>
+      <c r="D7" t="n">
+        <v>91</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1">
+        <f>IFERROR(E7/D7,0)</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>IF(D7&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-07-08 13:00
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -673,6 +673,33 @@
       </c>
       <c r="G7">
         <f>IF(D7&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="n">
+        <v>9960</v>
+      </c>
+      <c r="D8" t="n">
+        <v>46</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="1">
+        <f>IFERROR(E8/D8,0)</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>IF(D8&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-07-09 13:23
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -700,6 +700,33 @@
       </c>
       <c r="G8">
         <f>IF(D8&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>9986</v>
+      </c>
+      <c r="D9" t="n">
+        <v>26</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="1">
+        <f>IFERROR(E9/D9,0)</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>IF(D9&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-07-10 13:00
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -727,6 +727,33 @@
       </c>
       <c r="G9">
         <f>IF(D9&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10052</v>
+      </c>
+      <c r="D10" t="n">
+        <v>66</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="1">
+        <f>IFERROR(E10/D10,0)</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>IF(D10&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-07-11 13:00
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -754,6 +754,33 @@
       </c>
       <c r="G10">
         <f>IF(D10&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" t="n">
+        <v>10080</v>
+      </c>
+      <c r="D11" t="n">
+        <v>28</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="1">
+        <f>IFERROR(E11/D11,0)</f>
+        <v/>
+      </c>
+      <c r="G11">
+        <f>IF(D11&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-07-12 13:02
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -781,6 +781,33 @@
       </c>
       <c r="G11">
         <f>IF(D11&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>10110</v>
+      </c>
+      <c r="D12" t="n">
+        <v>30</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1">
+        <f>IFERROR(E12/D12,0)</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>IF(D12&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-07-26 13:06
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -808,6 +808,33 @@
       </c>
       <c r="G12">
         <f>IF(D12&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" t="n">
+        <v>10695</v>
+      </c>
+      <c r="D13" t="n">
+        <v>47</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1">
+        <f>IFERROR(E13/D13,0)</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>IF(D13&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-07-27 13:42
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -835,6 +835,33 @@
       </c>
       <c r="G13">
         <f>IF(D13&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" t="n">
+        <v>10776</v>
+      </c>
+      <c r="D14" t="n">
+        <v>81</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="1">
+        <f>IFERROR(E14/D14,0)</f>
+        <v/>
+      </c>
+      <c r="G14">
+        <f>IF(D14&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-07-28 13:11
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -862,6 +862,33 @@
       </c>
       <c r="G14">
         <f>IF(D14&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="n">
+        <v>10816</v>
+      </c>
+      <c r="D15" t="n">
+        <v>40</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="1">
+        <f>IFERROR(E15/D15,0)</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>IF(D15&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-02 13:57
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -889,6 +889,33 @@
       </c>
       <c r="G15">
         <f>IF(D15&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="n">
+        <v>10832</v>
+      </c>
+      <c r="D16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="1">
+        <f>IFERROR(E16/D16,0)</f>
+        <v/>
+      </c>
+      <c r="G16">
+        <f>IF(D16&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-06 13:15
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -916,6 +916,33 @@
       </c>
       <c r="G16">
         <f>IF(D16&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>10968</v>
+      </c>
+      <c r="D17" t="n">
+        <v>22</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="1">
+        <f>IFERROR(E17/D17,0)</f>
+        <v/>
+      </c>
+      <c r="G17">
+        <f>IF(D17&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-07 13:11
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -943,6 +943,33 @@
       </c>
       <c r="G17">
         <f>IF(D17&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C18" t="n">
+        <v>10997</v>
+      </c>
+      <c r="D18" t="n">
+        <v>29</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1">
+        <f>IFERROR(E18/D18,0)</f>
+        <v/>
+      </c>
+      <c r="G18">
+        <f>IF(D18&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-08 13:31
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -970,6 +970,33 @@
       </c>
       <c r="G18">
         <f>IF(D18&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C19" t="n">
+        <v>11033</v>
+      </c>
+      <c r="D19" t="n">
+        <v>36</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="1">
+        <f>IFERROR(E19/D19,0)</f>
+        <v/>
+      </c>
+      <c r="G19">
+        <f>IF(D19&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-09 13:10
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -997,6 +997,33 @@
       </c>
       <c r="G19">
         <f>IF(D19&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>11049</v>
+      </c>
+      <c r="D20" t="n">
+        <v>16</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="1">
+        <f>IFERROR(E20/D20,0)</f>
+        <v/>
+      </c>
+      <c r="G20">
+        <f>IF(D20&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-11 13:53
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1024,6 +1024,33 @@
       </c>
       <c r="G20">
         <f>IF(D20&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>11157</v>
+      </c>
+      <c r="D21" t="n">
+        <v>51</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="1">
+        <f>IFERROR(E21/D21,0)</f>
+        <v/>
+      </c>
+      <c r="G21">
+        <f>IF(D21&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-12 13:49
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1051,6 +1051,33 @@
       </c>
       <c r="G21">
         <f>IF(D21&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>11195</v>
+      </c>
+      <c r="D22" t="n">
+        <v>38</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="1">
+        <f>IFERROR(E22/D22,0)</f>
+        <v/>
+      </c>
+      <c r="G22">
+        <f>IF(D22&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-14 13:54
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1078,6 +1078,33 @@
       </c>
       <c r="G22">
         <f>IF(D22&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>11245</v>
+      </c>
+      <c r="D23" t="n">
+        <v>37</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="1">
+        <f>IFERROR(E23/D23,0)</f>
+        <v/>
+      </c>
+      <c r="G23">
+        <f>IF(D23&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-15 13:21
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1105,6 +1105,33 @@
       </c>
       <c r="G23">
         <f>IF(D23&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C24" t="n">
+        <v>11263</v>
+      </c>
+      <c r="D24" t="n">
+        <v>18</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="1">
+        <f>IFERROR(E24/D24,0)</f>
+        <v/>
+      </c>
+      <c r="G24">
+        <f>IF(D24&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-16 13:19
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1132,6 +1132,33 @@
       </c>
       <c r="G24">
         <f>IF(D24&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>11298</v>
+      </c>
+      <c r="D25" t="n">
+        <v>35</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="1">
+        <f>IFERROR(E25/D25,0)</f>
+        <v/>
+      </c>
+      <c r="G25">
+        <f>IF(D25&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-17 13:28
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1159,6 +1159,33 @@
       </c>
       <c r="G25">
         <f>IF(D25&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C26" t="n">
+        <v>11340</v>
+      </c>
+      <c r="D26" t="n">
+        <v>42</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="1">
+        <f>IFERROR(E26/D26,0)</f>
+        <v/>
+      </c>
+      <c r="G26">
+        <f>IF(D26&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -1173,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1373,6 +1400,62 @@
       </c>
       <c r="F7">
         <f>IF(D7&gt;=E7,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-W32</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Lyla</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <f>Settings!$B$4</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>IF(D8&gt;=E8,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-W32</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Cece</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <f>Settings!$B$4</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>IF(D9&gt;=E9,"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -1387,7 +1470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1561,6 +1644,54 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-W32</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Lyla</t>
+        </is>
+      </c>
+      <c r="C8">
+        <f>SUMIFS('Shoutouts Daily'!D:D,'Shoutouts Daily'!B:B,A8,'Shoutouts Daily'!C:C,B8)</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>Settings!$B$4</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>COUNTIFS('Shoutouts Daily'!B:B,A8,'Shoutouts Daily'!C:C,B8,'Shoutouts Daily'!D:D,"&gt;="&amp;D8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-W32</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Cece</t>
+        </is>
+      </c>
+      <c r="C9">
+        <f>SUMIFS('Shoutouts Daily'!D:D,'Shoutouts Daily'!B:B,A9,'Shoutouts Daily'!C:C,B9)</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>Settings!$B$4</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>COUNTIFS('Shoutouts Daily'!B:B,A9,'Shoutouts Daily'!C:C,B9,'Shoutouts Daily'!D:D,"&gt;="&amp;D9)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ratings 2026-08-18 13:04
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1186,6 +1186,33 @@
       </c>
       <c r="G26">
         <f>IF(D26&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C27" t="n">
+        <v>11411</v>
+      </c>
+      <c r="D27" t="n">
+        <v>71</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="1">
+        <f>IFERROR(E27/D27,0)</f>
+        <v/>
+      </c>
+      <c r="G27">
+        <f>IF(D27&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-19 13:03
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1213,6 +1213,33 @@
       </c>
       <c r="G27">
         <f>IF(D27&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C28" t="n">
+        <v>11467</v>
+      </c>
+      <c r="D28" t="n">
+        <v>56</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="1">
+        <f>IFERROR(E28/D28,0)</f>
+        <v/>
+      </c>
+      <c r="G28">
+        <f>IF(D28&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-20 13:05
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1240,6 +1240,33 @@
       </c>
       <c r="G28">
         <f>IF(D28&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C29" t="n">
+        <v>11492</v>
+      </c>
+      <c r="D29" t="n">
+        <v>25</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="1">
+        <f>IFERROR(E29/D29,0)</f>
+        <v/>
+      </c>
+      <c r="G29">
+        <f>IF(D29&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-21 13:04
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1267,6 +1267,33 @@
       </c>
       <c r="G29">
         <f>IF(D29&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C30" t="n">
+        <v>11514</v>
+      </c>
+      <c r="D30" t="n">
+        <v>22</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="1">
+        <f>IFERROR(E30/D30,0)</f>
+        <v/>
+      </c>
+      <c r="G30">
+        <f>IF(D30&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-22 13:30
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1294,6 +1294,33 @@
       </c>
       <c r="G30">
         <f>IF(D30&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>11537</v>
+      </c>
+      <c r="D31" t="n">
+        <v>23</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="1">
+        <f>IFERROR(E31/D31,0)</f>
+        <v/>
+      </c>
+      <c r="G31">
+        <f>IF(D31&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-23 13:04
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1321,6 +1321,33 @@
       </c>
       <c r="G31">
         <f>IF(D31&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>11564</v>
+      </c>
+      <c r="D32" t="n">
+        <v>27</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="1">
+        <f>IFERROR(E32/D32,0)</f>
+        <v/>
+      </c>
+      <c r="G32">
+        <f>IF(D32&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-24 13:25
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1348,6 +1348,33 @@
       </c>
       <c r="G32">
         <f>IF(D32&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>11620</v>
+      </c>
+      <c r="D33" t="n">
+        <v>56</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="1">
+        <f>IFERROR(E33/D33,0)</f>
+        <v/>
+      </c>
+      <c r="G33">
+        <f>IF(D33&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-25 13:06
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1375,6 +1375,33 @@
       </c>
       <c r="G33">
         <f>IF(D33&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>11685</v>
+      </c>
+      <c r="D34" t="n">
+        <v>65</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="1">
+        <f>IFERROR(E34/D34,0)</f>
+        <v/>
+      </c>
+      <c r="G34">
+        <f>IF(D34&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-26 13:12
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1402,6 +1402,33 @@
       </c>
       <c r="G34">
         <f>IF(D34&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>11721</v>
+      </c>
+      <c r="D35" t="n">
+        <v>36</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="1">
+        <f>IFERROR(E35/D35,0)</f>
+        <v/>
+      </c>
+      <c r="G35">
+        <f>IF(D35&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-08-30 13:00
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1429,6 +1429,33 @@
       </c>
       <c r="G35">
         <f>IF(D35&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>11896</v>
+      </c>
+      <c r="D36" t="n">
+        <v>69</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="1">
+        <f>IFERROR(E36/D36,0)</f>
+        <v/>
+      </c>
+      <c r="G36">
+        <f>IF(D36&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-09-02 13:37
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1456,6 +1456,33 @@
       </c>
       <c r="G36">
         <f>IF(D36&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>12061</v>
+      </c>
+      <c r="D37" t="n">
+        <v>60</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="1">
+        <f>IFERROR(E37/D37,0)</f>
+        <v/>
+      </c>
+      <c r="G37">
+        <f>IF(D37&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-09-03 13:52
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1483,6 +1483,33 @@
       </c>
       <c r="G37">
         <f>IF(D37&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>12102</v>
+      </c>
+      <c r="D38" t="n">
+        <v>41</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="1">
+        <f>IFERROR(E38/D38,0)</f>
+        <v/>
+      </c>
+      <c r="G38">
+        <f>IF(D38&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-09-04 13:30
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1510,6 +1510,33 @@
       </c>
       <c r="G38">
         <f>IF(D38&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>12149</v>
+      </c>
+      <c r="D39" t="n">
+        <v>47</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="1">
+        <f>IFERROR(E39/D39,0)</f>
+        <v/>
+      </c>
+      <c r="G39">
+        <f>IF(D39&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ratings 2026-09-08 13:57
</commit_message>
<xml_diff>
--- a/data/logs/Avis_Dashboard_Log.xlsx
+++ b/data/logs/Avis_Dashboard_Log.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1537,6 +1537,33 @@
       </c>
       <c r="G39">
         <f>IF(D39&gt;=Settings!$B$3,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C40" t="n">
+        <v>12309</v>
+      </c>
+      <c r="D40" t="n">
+        <v>42</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="1">
+        <f>IFERROR(E40/D40,0)</f>
+        <v/>
+      </c>
+      <c r="G40">
+        <f>IF(D40&gt;=Settings!$B$3,"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>